<commit_message>
20260629: Outlook to Confluence folder structure created, but failed - 폴더 생성 안됨
</commit_message>
<xml_diff>
--- a/Python_2026/KPI_Measurement/AnD_KPI_2026.xlsx
+++ b/Python_2026/KPI_Measurement/AnD_KPI_2026.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\_Development_2026\Python_2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\_Development_2026\Python_2026\KPI_Measurement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38FC4A28-244A-43AE-841C-78FA7C12F4A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D573F5C8-5755-4310-BC2C-5DD5A6D84F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2145" yWindow="600" windowWidth="25725" windowHeight="14235" xr2:uid="{53B19080-9F04-48C2-B8B2-0D660C2AD9E9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{53B19080-9F04-48C2-B8B2-0D660C2AD9E9}"/>
   </bookViews>
   <sheets>
     <sheet name="export" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" concurrentManualCount="12"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -30,6 +30,99 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="2">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <futureMetadata name="XLRICHVALUE" count="3">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="1"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="2"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+  <valueMetadata count="3">
+    <bk>
+      <rc t="2" v="0"/>
+    </bk>
+    <bk>
+      <rc t="2" v="1"/>
+    </bk>
+    <bk>
+      <rc t="2" v="2"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
+<file path=xl/python.xml><?xml version="1.0" encoding="utf-8"?>
+<python xmlns="http://schemas.microsoft.com/office/spreadsheetml/2023/python">
+  <environmentDefinition id="{882DD1B0-6546-4DFA-8A08-902A380B44EA}">
+    <initialization userModified="1">
+      <code xml:space="preserve">import numpy as np
+import pandas as pd
+import matplotlib.pyplot as plt
+import seaborn as sns
+import statsmodels as sm
+import excel
+import warnings
+warnings.simplefilter('ignore')
+excel.set_xl_scalar_conversion(excel.convert_to_scalar)
+excel.set_xl_array_conversion(excel.convert_to_dataframe)
+</code>
+    </initialization>
+  </environmentDefinition>
+  <pythonScripts>
+    <pythonScript>
+      <code>import pandas as pd
+# M값만 사용
+df = pd.DataFrame({
+    "M": [xl(%P2%)]
+})
+# Step 1: 구간 정의 (기존 C 기준 재활용)
+bins = [-1, 0, 2, 5, 9, 12, float('inf')]
+scores = [0, 0.5, 1, 1.5, 2, 2.5]
+# Step 2: Pandas cut으로 점수 매핑
+df["score"] = pd.cut(df["M"], bins=bins, labels=scores).astype(float)
+# 결과 반환
+df["score"].iloc[0]</code>
+    </pythonScript>
+  </pythonScripts>
+</python>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -873,14 +966,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -1160,6 +1253,9 @@
                 <c:pt idx="4">
                   <c:v>0.1951219512195122</c:v>
                 </c:pt>
+                <c:pt idx="5">
+                  <c:v>9.7560975609756101E-2</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -1311,6 +1407,9 @@
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0.72727272727272729</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.84848484848484851</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3587,16 +3686,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>493568</xdr:colOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>60613</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>266700</xdr:rowOff>
+      <xdr:rowOff>284018</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>658091</xdr:colOff>
+      <xdr:col>33</xdr:col>
+      <xdr:colOff>432955</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>190501</xdr:rowOff>
+      <xdr:rowOff>207819</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3622,6 +3721,109 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="3">
+  <rv s="0">
+    <fb>1</fb>
+    <v>&lt;class 'numpy.float64'&gt;</v>
+    <v>float64</v>
+    <v>1.0</v>
+    <v>1</v>
+    <v>0</v>
+  </rv>
+  <rv s="0">
+    <fb>0</fb>
+    <v>&lt;class 'numpy.float64'&gt;</v>
+    <v>float64</v>
+    <v>0.0</v>
+    <v>0</v>
+    <v>0</v>
+  </rv>
+  <rv s="0">
+    <fb>0.5</fb>
+    <v>&lt;class 'numpy.float64'&gt;</v>
+    <v>float64</v>
+    <v>0.5</v>
+    <v>0.5</v>
+    <v>0</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_python">
+    <k n="Python_type" t="s"/>
+    <k n="Python_typeName" t="s"/>
+    <k n="Python_str" t="s"/>
+    <k n="basicValue"/>
+    <k n="_Provider" t="spb"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/rdsupportingpropertybag.xml><?xml version="1.0" encoding="utf-8"?>
+<supportingPropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2">
+  <spbData count="1">
+    <spb s="0">
+      <v>https://www.anaconda.com/excel</v>
+      <v>https://res.cdn.office.net/officepysvc/prod-service/anacondalogo.png</v>
+      <v>Python provided by Anaconda</v>
+    </spb>
+  </spbData>
+</supportingPropertyBags>
+</file>
+
+<file path=xl/richData/rdsupportingpropertybagstructure.xml><?xml version="1.0" encoding="utf-8"?>
+<spbStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" count="1">
+  <s>
+    <k n="link" t="s"/>
+    <k n="logo" t="s"/>
+    <k n="name" t="s"/>
+  </s>
+</spbStructures>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4076,6 +4278,13 @@
       <c r="L2" s="7">
         <v>1.5</v>
       </c>
+      <c r="M2" s="7">
+        <v>3</v>
+      </c>
+      <c r="N2" s="7" cm="1" vm="1">
+        <f t="array" ref="N2">_xlfn._xlws.PY(0,1,M2)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="3" spans="1:28" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
@@ -4114,9 +4323,16 @@
       <c r="L3" s="7">
         <v>0.5</v>
       </c>
+      <c r="M3" s="7">
+        <v>0</v>
+      </c>
+      <c r="N3" s="7" cm="1" vm="2">
+        <f t="array" ref="N3">_xlfn._xlws.PY(0,1,M3)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="4" spans="1:28" ht="82.5" x14ac:dyDescent="0.3">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="10" t="s">
         <v>14</v>
       </c>
       <c r="B4" s="7" t="s">
@@ -4150,6 +4366,13 @@
         <v>1</v>
       </c>
       <c r="L4" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="M4" s="7">
+        <v>2</v>
+      </c>
+      <c r="N4" s="7" cm="1" vm="3">
+        <f t="array" ref="N4">_xlfn._xlws.PY(0,1,M4)</f>
         <v>0.5</v>
       </c>
     </row>
@@ -4190,9 +4413,16 @@
       <c r="L5" s="7">
         <v>0.5</v>
       </c>
+      <c r="M5" s="7">
+        <v>0</v>
+      </c>
+      <c r="N5" s="7" cm="1" vm="2">
+        <f t="array" ref="N5">_xlfn._xlws.PY(0,1,M5)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:28" ht="66" x14ac:dyDescent="0.3">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="10" t="s">
         <v>16</v>
       </c>
       <c r="B6" s="7" t="s">
@@ -4227,6 +4457,13 @@
       </c>
       <c r="L6" s="7">
         <v>0.5</v>
+      </c>
+      <c r="M6" s="7">
+        <v>3</v>
+      </c>
+      <c r="N6" s="7" cm="1" vm="1">
+        <f t="array" ref="N6">_xlfn._xlws.PY(0,1,M6)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:28" ht="82.5" x14ac:dyDescent="0.3">
@@ -4266,9 +4503,16 @@
       <c r="L7" s="7">
         <v>0</v>
       </c>
+      <c r="M7" s="7">
+        <v>0</v>
+      </c>
+      <c r="N7" s="7" cm="1" vm="2">
+        <f t="array" ref="N7">_xlfn._xlws.PY(0,1,M7)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:28" ht="82.5" x14ac:dyDescent="0.3">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="10" t="s">
         <v>21</v>
       </c>
       <c r="B8" s="7" t="s">
@@ -4304,9 +4548,16 @@
       <c r="L8" s="7">
         <v>0.5</v>
       </c>
+      <c r="M8" s="7">
+        <v>0</v>
+      </c>
+      <c r="N8" s="7" cm="1" vm="2">
+        <f t="array" ref="N8">_xlfn._xlws.PY(0,1,M8)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:28" ht="115.5" x14ac:dyDescent="0.3">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="10" t="s">
         <v>22</v>
       </c>
       <c r="B9" s="7" t="s">
@@ -4341,6 +4592,13 @@
       </c>
       <c r="L9" s="7">
         <v>0.5</v>
+      </c>
+      <c r="M9" s="7">
+        <v>0</v>
+      </c>
+      <c r="N9" s="7" cm="1" vm="2">
+        <f t="array" ref="N9">_xlfn._xlws.PY(0,1,M9)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.3">
@@ -4355,30 +4613,45 @@
         <v>16.5</v>
       </c>
       <c r="E10" s="7">
+        <f t="shared" ref="E10:N10" si="0">SUM(E2:E9)</f>
         <v>11</v>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="7">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="G10" s="7">
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="7">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="I10" s="7">
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="J10" s="5">
+      <c r="J10" s="7">
+        <f t="shared" si="0"/>
         <v>4.5</v>
       </c>
       <c r="K10" s="7">
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="L10" s="5">
+      <c r="L10" s="7">
+        <f t="shared" si="0"/>
         <v>4.5</v>
       </c>
-      <c r="N10" s="2"/>
+      <c r="M10" s="7">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="N10" s="7">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
       <c r="P10" s="2"/>
       <c r="R10" s="2"/>
       <c r="T10" s="2"/>
@@ -4420,12 +4693,20 @@
         <f>1-(L10/$D$10)</f>
         <v>0.72727272727272729</v>
       </c>
+      <c r="M11" s="6">
+        <f>(M10/$C$10)</f>
+        <v>9.7560975609756101E-2</v>
+      </c>
+      <c r="N11" s="6">
+        <f>1-(N10/$D$10)</f>
+        <v>0.84848484848484851</v>
+      </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="D13" s="10"/>
+      <c r="D13" s="11"/>
       <c r="E13" s="4" t="s">
         <v>34</v>
       </c>
@@ -4467,10 +4748,10 @@
       </c>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="D14" s="11"/>
+      <c r="D14" s="12"/>
       <c r="E14" s="6">
         <f>(E10/$C$10)</f>
         <v>0.13414634146341464</v>
@@ -4487,7 +4768,10 @@
         <f>(K10/$C$10)</f>
         <v>0.1951219512195122</v>
       </c>
-      <c r="I14" s="6"/>
+      <c r="I14" s="6">
+        <f>(M10/$C$10)</f>
+        <v>9.7560975609756101E-2</v>
+      </c>
       <c r="J14" s="6"/>
       <c r="K14" s="5"/>
       <c r="L14" s="5"/>
@@ -4497,14 +4781,14 @@
       <c r="P14" s="5"/>
       <c r="Q14" s="3">
         <f>AVERAGE(E14:P14)</f>
-        <v>0.21646341463414637</v>
+        <v>0.1926829268292683</v>
       </c>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="C15" s="11" t="s">
+      <c r="C15" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="D15" s="11"/>
+      <c r="D15" s="12"/>
       <c r="E15" s="6">
         <f>1-(F10/$D$10)</f>
         <v>0.81818181818181812</v>
@@ -4521,7 +4805,10 @@
         <f>1-(L10/$D$10)</f>
         <v>0.72727272727272729</v>
       </c>
-      <c r="I15" s="5"/>
+      <c r="I15" s="6">
+        <f>1-(N10/$D$10)</f>
+        <v>0.84848484848484851</v>
+      </c>
       <c r="J15" s="5"/>
       <c r="K15" s="5"/>
       <c r="L15" s="5"/>
@@ -4531,7 +4818,7 @@
       <c r="P15" s="5"/>
       <c r="Q15" s="3">
         <f>AVERAGE(E15:P15)</f>
-        <v>0.75757575757575757</v>
+        <v>0.77575757575757576</v>
       </c>
     </row>
   </sheetData>

</xml_diff>